<commit_message>
Project Coding Structre, per every team member
</commit_message>
<xml_diff>
--- a/Documentation/02_System Design/00_System_Design_Master/System_Design_Decision_Register.xlsx
+++ b/Documentation/02_System Design/00_System_Design_Master/System_Design_Decision_Register.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BCY 4th Year\MP Online\AI-ITSM\Documentation\02_System Design\00_System_Design_Master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38376D5-08C9-40CE-B3CB-FF2B08027EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C268F2AF-45E2-4DCA-B92C-13A76A1C8717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="76">
   <si>
     <t>ID</t>
   </si>
@@ -112,6 +112,147 @@
   </si>
   <si>
     <t>To validate</t>
+  </si>
+  <si>
+    <t>SD-005</t>
+  </si>
+  <si>
+    <t>SD-006</t>
+  </si>
+  <si>
+    <t>SD-007</t>
+  </si>
+  <si>
+    <t>SD-008</t>
+  </si>
+  <si>
+    <t>ASP.NET Core Web API where appropriate</t>
+  </si>
+  <si>
+    <t>Proposed</t>
+  </si>
+  <si>
+    <t>Possible</t>
+  </si>
+  <si>
+    <t>SD-009</t>
+  </si>
+  <si>
+    <t>SD-010</t>
+  </si>
+  <si>
+    <t>SD-011</t>
+  </si>
+  <si>
+    <t>SD-012</t>
+  </si>
+  <si>
+    <t>Role-based authorization</t>
+  </si>
+  <si>
+    <t>SD-013</t>
+  </si>
+  <si>
+    <t>SD-014</t>
+  </si>
+  <si>
+    <t>Faculty instruction + AR-01–AR-06</t>
+  </si>
+  <si>
+    <t>SD-015</t>
+  </si>
+  <si>
+    <t>Unresolved</t>
+  </si>
+  <si>
+    <t>C# as primary programming language</t>
+  </si>
+  <si>
+    <t>Project technology direction</t>
+  </si>
+  <si>
+    <t>Required application development direction</t>
+  </si>
+  <si>
+    <t>ASP.NET Core as application framework</t>
+  </si>
+  <si>
+    <t>Provides the C# web application framework</t>
+  </si>
+  <si>
+    <t>ASP.NET Core MVC with Razor/CSHTML for web UI</t>
+  </si>
+  <si>
+    <t>Current implementation direction</t>
+  </si>
+  <si>
+    <t>Provides the server-rendered web interface for the system</t>
+  </si>
+  <si>
+    <t>No direct impact</t>
+  </si>
+  <si>
+    <t>Current architecture direction</t>
+  </si>
+  <si>
+    <t>Provides API-based communication where required</t>
+  </si>
+  <si>
+    <t>Entity Framework Core for data access</t>
+  </si>
+  <si>
+    <t>Current technology direction</t>
+  </si>
+  <si>
+    <t>Provides ORM-based access to the relational database</t>
+  </si>
+  <si>
+    <t>SQL Server as relational database</t>
+  </si>
+  <si>
+    <t>Current technology direction + Database v1</t>
+  </si>
+  <si>
+    <t>Directly compatible with the existing SQL Server-oriented Database v1</t>
+  </si>
+  <si>
+    <t>ASP.NET Core Identity for authentication/identity</t>
+  </si>
+  <si>
+    <t>Proposed / Requires validation</t>
+  </si>
+  <si>
+    <t>Provides authentication and identity management, but must be reconciled with Database v1 Users/Roles</t>
+  </si>
+  <si>
+    <t>Requirement Analysis NFR-06, NFR-07 + technology direction</t>
+  </si>
+  <si>
+    <t>Supports role-restricted functionality and administration</t>
+  </si>
+  <si>
+    <t>Gemini API for AI capabilities</t>
+  </si>
+  <si>
+    <t>Proposed implementation technology for the AI requirements</t>
+  </si>
+  <si>
+    <t>n8n for automation</t>
+  </si>
+  <si>
+    <t>Faculty-provided direction</t>
+  </si>
+  <si>
+    <t>Faculty has specified n8n for the project's automation</t>
+  </si>
+  <si>
+    <t>Background-processing mechanism</t>
+  </si>
+  <si>
+    <t>Requirement Analysis NFR-04, NFR-11</t>
+  </si>
+  <si>
+    <t>Exact mechanism has not yet been decided</t>
   </si>
 </sst>
 </file>
@@ -155,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -167,6 +308,9 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -449,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="12.77734375" customWidth="1"/>
@@ -564,7 +708,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>23</v>
       </c>
@@ -588,6 +732,292 @@
       </c>
       <c r="H5" s="4" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="2">
+        <v>2</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="2">
+        <v>2</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="2">
+        <v>2</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="2">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="2">
+        <v>2</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="2">
+        <v>2</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>